<commit_message>
add draw & stack navigation
</commit_message>
<xml_diff>
--- a/CPA_FSD_Reskill_5_Week_Learning_Plan.xlsx
+++ b/CPA_FSD_Reskill_5_Week_Learning_Plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\learning\React\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B152376E-BAF0-48D3-BCC6-064D8860511E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BCB9993-1EAB-4831-BBB2-7AE62D59C15F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="917" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,6 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly Summary'!$A$1:$D$6</definedName>
   </definedNames>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -1418,7 +1419,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="s">
-        <v>11</v>
+        <v>148</v>
       </c>
       <c r="F24">
         <v>3</v>
@@ -1441,7 +1442,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="s">
-        <v>11</v>
+        <v>148</v>
       </c>
       <c r="F25">
         <v>3</v>
@@ -1464,7 +1465,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="s">
-        <v>11</v>
+        <v>148</v>
       </c>
       <c r="F26">
         <v>4</v>

</xml_diff>

<commit_message>
add i18next to expo demo
</commit_message>
<xml_diff>
--- a/CPA_FSD_Reskill_5_Week_Learning_Plan.xlsx
+++ b/CPA_FSD_Reskill_5_Week_Learning_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\learning\React\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3784D2FE-A9F1-4396-9681-5A0897A727C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D345352-900C-45C0-8405-FC8E250DAC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="917" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="152">
   <si>
     <t>Week</t>
   </si>
@@ -228,15 +228,9 @@
     <t>State and Hooks</t>
   </si>
   <si>
-    <t>Connect mobile app to API</t>
-  </si>
-  <si>
     <t>Forms and validation</t>
   </si>
   <si>
-    <t>Mobile input and validation</t>
-  </si>
-  <si>
     <t>Authentication</t>
   </si>
   <si>
@@ -481,6 +475,29 @@
   </si>
   <si>
     <t>Apply React knowledge to RN,无localstorage概念</t>
+  </si>
+  <si>
+    <t>Connect mobile app to API, 使用axios一样</t>
+  </si>
+  <si>
+    <t>Mobile input and validation， react hook form + zod（定义字段和映射）</t>
+  </si>
+  <si>
+    <t>// 3. 初始化 react-hook-form
+  const {
+    control,
+    handleSubmit,
+    reset,
+    formState: { errors, isSubmitting },
+  } = useForm&lt;PostFormData&gt;({
+    resolver: zodResolver(postSchema),
+    defaultValues: {
+      title: '',
+      body: '',
+      userId: '1',
+    },
+    mode: 'onBlur',
+  });</t>
   </si>
 </sst>
 </file>
@@ -542,12 +559,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -869,8 +890,8 @@
     <col min="3" max="3" width="41" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="44" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" customWidth="1"/>
+    <col min="7" max="7" width="45.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -889,7 +910,7 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -910,7 +931,7 @@
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F2">
         <v>4</v>
@@ -933,7 +954,7 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F3">
         <v>4</v>
@@ -956,7 +977,7 @@
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F4">
         <v>2</v>
@@ -979,7 +1000,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F5">
         <v>3</v>
@@ -1002,7 +1023,7 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F6">
         <v>3</v>
@@ -1025,7 +1046,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F7">
         <v>4</v>
@@ -1048,7 +1069,7 @@
         <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F8">
         <v>3</v>
@@ -1071,7 +1092,7 @@
         <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F9">
         <v>2</v>
@@ -1094,7 +1115,7 @@
         <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F10">
         <v>4</v>
@@ -1117,7 +1138,7 @@
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F11" s="2">
         <v>6</v>
@@ -1140,7 +1161,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F12">
         <v>3</v>
@@ -1163,7 +1184,7 @@
         <v>10</v>
       </c>
       <c r="E13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F13">
         <v>3</v>
@@ -1186,7 +1207,7 @@
         <v>24</v>
       </c>
       <c r="E14" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F14">
         <v>2</v>
@@ -1209,7 +1230,7 @@
         <v>24</v>
       </c>
       <c r="E15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -1218,7 +1239,7 @@
         <v>40</v>
       </c>
       <c r="H15" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -1235,7 +1256,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -1244,7 +1265,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -1258,7 +1279,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -1267,7 +1288,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1281,7 +1302,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F18">
         <v>4</v>
@@ -1290,7 +1311,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -1304,7 +1325,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F19">
         <v>2</v>
@@ -1313,7 +1334,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1327,7 +1348,7 @@
         <v>24</v>
       </c>
       <c r="E20" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F20">
         <v>3</v>
@@ -1336,7 +1357,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>32</v>
       </c>
@@ -1350,7 +1371,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F21" s="2">
         <v>8</v>
@@ -1359,7 +1380,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -1373,7 +1394,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F22">
         <v>2</v>
@@ -1382,7 +1403,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -1396,7 +1417,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -1405,7 +1426,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>53</v>
       </c>
@@ -1419,7 +1440,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F24">
         <v>3</v>
@@ -1428,7 +1449,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -1442,7 +1463,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F25">
         <v>3</v>
@@ -1451,7 +1472,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>53</v>
       </c>
@@ -1465,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F26">
         <v>4</v>
@@ -1474,7 +1495,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -1488,16 +1509,16 @@
         <v>10</v>
       </c>
       <c r="E27" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F27">
         <v>3</v>
       </c>
       <c r="G27" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>53</v>
       </c>
@@ -1511,16 +1532,16 @@
         <v>10</v>
       </c>
       <c r="E28" t="s">
-        <v>11</v>
+        <v>145</v>
       </c>
       <c r="F28">
         <v>4</v>
       </c>
       <c r="G28" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>53</v>
       </c>
@@ -1528,7 +1549,7 @@
         <v>54</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
         <v>24</v>
@@ -1540,10 +1561,13 @@
         <v>3</v>
       </c>
       <c r="G29" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+        <v>150</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>53</v>
       </c>
@@ -1551,7 +1575,7 @@
         <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
         <v>10</v>
@@ -1563,10 +1587,10 @@
         <v>3</v>
       </c>
       <c r="G30" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>53</v>
       </c>
@@ -1574,7 +1598,7 @@
         <v>54</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D31" t="s">
         <v>24</v>
@@ -1586,10 +1610,10 @@
         <v>3</v>
       </c>
       <c r="G31" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>53</v>
       </c>
@@ -1597,7 +1621,7 @@
         <v>54</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>10</v>
@@ -1609,18 +1633,18 @@
         <v>6</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>73</v>
+      </c>
+      <c r="B33" t="s">
+        <v>74</v>
+      </c>
+      <c r="C33" t="s">
         <v>75</v>
-      </c>
-      <c r="B33" t="s">
-        <v>76</v>
-      </c>
-      <c r="C33" t="s">
-        <v>77</v>
       </c>
       <c r="D33" t="s">
         <v>10</v>
@@ -1632,18 +1656,18 @@
         <v>4</v>
       </c>
       <c r="G33" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C34" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D34" t="s">
         <v>10</v>
@@ -1655,18 +1679,18 @@
         <v>3</v>
       </c>
       <c r="G34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C35" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D35" t="s">
         <v>10</v>
@@ -1678,18 +1702,18 @@
         <v>4</v>
       </c>
       <c r="G35" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C36" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D36" t="s">
         <v>10</v>
@@ -1701,18 +1725,18 @@
         <v>3</v>
       </c>
       <c r="G36" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C37" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D37" t="s">
         <v>10</v>
@@ -1724,18 +1748,18 @@
         <v>4</v>
       </c>
       <c r="G37" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C38" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D38" t="s">
         <v>10</v>
@@ -1747,18 +1771,18 @@
         <v>4</v>
       </c>
       <c r="G38" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C39" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D39" t="s">
         <v>10</v>
@@ -1770,18 +1794,18 @@
         <v>4</v>
       </c>
       <c r="G39" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C40" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D40" t="s">
         <v>10</v>
@@ -1793,18 +1817,18 @@
         <v>3</v>
       </c>
       <c r="G40" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C41" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D41" t="s">
         <v>24</v>
@@ -1816,18 +1840,18 @@
         <v>2</v>
       </c>
       <c r="G41" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B42" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C42" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D42" t="s">
         <v>10</v>
@@ -1839,18 +1863,18 @@
         <v>6</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B43" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C43" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D43" t="s">
         <v>24</v>
@@ -1862,18 +1886,18 @@
         <v>4</v>
       </c>
       <c r="G43" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B44" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C44" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D44" t="s">
         <v>24</v>
@@ -1885,18 +1909,18 @@
         <v>4</v>
       </c>
       <c r="G44" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>24</v>
@@ -1908,18 +1932,18 @@
         <v>4</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
+        <v>102</v>
+      </c>
+      <c r="B46" t="s">
+        <v>103</v>
+      </c>
+      <c r="C46" t="s">
         <v>104</v>
-      </c>
-      <c r="B46" t="s">
-        <v>105</v>
-      </c>
-      <c r="C46" t="s">
-        <v>106</v>
       </c>
       <c r="D46" t="s">
         <v>10</v>
@@ -1931,18 +1955,18 @@
         <v>5</v>
       </c>
       <c r="G46" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B47" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C47" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
@@ -1954,18 +1978,18 @@
         <v>4</v>
       </c>
       <c r="G47" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B48" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C48" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D48" t="s">
         <v>10</v>
@@ -1977,18 +2001,18 @@
         <v>4</v>
       </c>
       <c r="G48" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B49" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C49" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D49" t="s">
         <v>10</v>
@@ -2000,18 +2024,18 @@
         <v>2</v>
       </c>
       <c r="G49" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B50" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C50" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D50" t="s">
         <v>24</v>
@@ -2023,18 +2047,18 @@
         <v>2</v>
       </c>
       <c r="G50" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B51" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C51" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D51" t="s">
         <v>24</v>
@@ -2046,18 +2070,18 @@
         <v>2</v>
       </c>
       <c r="G51" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B52" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C52" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D52" t="s">
         <v>24</v>
@@ -2069,18 +2093,18 @@
         <v>3</v>
       </c>
       <c r="G52" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B53" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C53" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D53" t="s">
         <v>10</v>
@@ -2092,18 +2116,18 @@
         <v>10</v>
       </c>
       <c r="G53" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B54" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C54" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D54" t="s">
         <v>24</v>
@@ -2115,7 +2139,7 @@
         <v>3</v>
       </c>
       <c r="G54" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2146,10 +2170,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>5</v>
@@ -2160,10 +2184,10 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D2">
         <v>35</v>
@@ -2174,10 +2198,10 @@
         <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D3">
         <v>35</v>
@@ -2191,7 +2215,7 @@
         <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D4">
         <v>37</v>
@@ -2199,13 +2223,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D5">
         <v>41</v>
@@ -2213,13 +2237,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D6">
         <v>35</v>
@@ -2246,10 +2270,10 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -2257,13 +2281,13 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -2271,7 +2295,7 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -2282,7 +2306,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -2293,60 +2317,60 @@
         <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B8" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>